<commit_message>
Contracts report add status
</commit_message>
<xml_diff>
--- a/app/templates/report/contratos.xlsx
+++ b/app/templates/report/contratos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\oimbra\custom\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C98A29-2849-449A-B4C3-C7D7C0FD1BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C2D332-084B-421D-BB97-11EB03A8E552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Contratos" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Contratos!$A$2:$L$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Contratos!$A$2:$M$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>Contratos</t>
   </si>
@@ -578,28 +578,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="48.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" style="1" customWidth="1"/>
-    <col min="8" max="9" width="41.85546875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15" style="1" customWidth="1"/>
-    <col min="11" max="11" width="21.28515625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="37" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="24.85546875" style="1"/>
+    <col min="3" max="3" width="20.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="48.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" style="1" customWidth="1"/>
+    <col min="9" max="10" width="41.85546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15" style="1" customWidth="1"/>
+    <col min="12" max="12" width="21.28515625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="37" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="24.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="5" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" s="5" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
@@ -607,54 +608,58 @@
         <v>2</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="6"/>
       <c r="E2" s="6"/>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="K2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="L2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="M2" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="F3" s="3"/>
       <c r="G3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="3"/>
+      <c r="H3" s="7" t="s">
+        <v>7</v>
+      </c>
       <c r="I3" s="3"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8" t="s">
+      <c r="J3" s="3"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:L2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A2:M2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Contracts report add status v2
</commit_message>
<xml_diff>
--- a/app/templates/report/contratos.xlsx
+++ b/app/templates/report/contratos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\oimbra\custom\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C2D332-084B-421D-BB97-11EB03A8E552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B15CFA11-9517-431E-9678-7E870FF28E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -582,7 +582,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.140625" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="48.5703125" style="1" customWidth="1"/>

</xml_diff>